<commit_message>
Script aggiornati e snakefile funzionante
</commit_message>
<xml_diff>
--- a/flow_cytometry_db.xlsx
+++ b/flow_cytometry_db.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rossi\ASCAT_UMA\db_uma\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\anna_rossi\TESI_PROJECT\db_uma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959D0F21-BB36-4324-8EFC-441AD1A6BBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7B73C4-968F-431C-8372-71608373EA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
     <sheet name="db_purity_0.90" sheetId="2" r:id="rId2"/>
+    <sheet name="db_purity_no7500" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">metadata!$A$1:$N$931</definedName>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6580" uniqueCount="5249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6635" uniqueCount="5249">
   <si>
     <t>AIO_ID</t>
   </si>
@@ -57770,4 +57771,299 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21900F3-6116-4F5B-A4F5-6D05B8559A7A}">
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>5248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4492</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4493</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4494</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4495</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>4496</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4497</v>
+      </c>
+      <c r="H2" s="3">
+        <v>45762</v>
+      </c>
+      <c r="I2" s="4">
+        <v>51</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0.112</v>
+      </c>
+      <c r="K2" s="4">
+        <v>5111538</v>
+      </c>
+      <c r="L2" s="4">
+        <v>1998373</v>
+      </c>
+      <c r="M2" s="4">
+        <v>3113165</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O2" s="5">
+        <v>0.90400000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4516</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4517</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4518</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>4519</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>4520</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>4521</v>
+      </c>
+      <c r="H3" s="3">
+        <v>45734</v>
+      </c>
+      <c r="I3" s="4">
+        <v>51</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0.106</v>
+      </c>
+      <c r="K3" s="4">
+        <v>5514054</v>
+      </c>
+      <c r="L3" s="4">
+        <v>2240702</v>
+      </c>
+      <c r="M3" s="4">
+        <v>3273352</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O3" s="5">
+        <v>0.90700000000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>4742</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4743</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>4744</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>4745</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4746</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>4747</v>
+      </c>
+      <c r="H4" s="3">
+        <v>45831</v>
+      </c>
+      <c r="I4" s="4">
+        <v>58</v>
+      </c>
+      <c r="J4" s="4">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="K4" s="4">
+        <v>5077971</v>
+      </c>
+      <c r="L4" s="4">
+        <v>1466029</v>
+      </c>
+      <c r="M4" s="4">
+        <v>3611942</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" s="5">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>4754</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4755</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>4756</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>4757</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>4758</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>4759</v>
+      </c>
+      <c r="H5" s="3">
+        <v>45812</v>
+      </c>
+      <c r="I5" s="4">
+        <v>58</v>
+      </c>
+      <c r="J5" s="4">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="K5" s="4">
+        <v>5880890</v>
+      </c>
+      <c r="L5" s="4">
+        <v>1294664</v>
+      </c>
+      <c r="M5" s="4">
+        <v>4586226</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O5" s="5">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>5002</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5003</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>5004</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>5005</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>5006</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>5007</v>
+      </c>
+      <c r="H6" s="3">
+        <v>45971</v>
+      </c>
+      <c r="I6" s="4">
+        <v>66</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="K6" s="4">
+        <v>6385965</v>
+      </c>
+      <c r="L6" s="4">
+        <v>2508924</v>
+      </c>
+      <c r="M6" s="4">
+        <v>3877041</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O6" s="5">
+        <v>0.90900000000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>